<commit_message>
xlsform: emit question_head note before first likert item
Scales like GAD7 and PHQ9 store a global instruction string in
likert_options.question_head. The converter now emits this as a note
row before the first likert question, so the instruction appears in
the rendered form. Rebuilt affected sample files.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/xlsform_samples/GAD7.xlsx
+++ b/tools/xlsform_samples/GAD7.xlsx
@@ -442,11 +442,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -524,32 +524,24 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>select_one likert_main</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>gad1</t>
+          <t>question_head</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Feeling nervous, anxious or on edge</t>
+          <t>Over the last 2 weeks, how often have you been bothered by the following problems?</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>likert</t>
-        </is>
-      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
@@ -563,12 +555,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>gad2</t>
+          <t>gad1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Not being able to stop or control worrying</t>
+          <t>Feeling nervous, anxious or on edge</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
@@ -597,12 +589,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>gad3</t>
+          <t>gad2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Worrying too much about different things</t>
+          <t>Not being able to stop or control worrying</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -631,12 +623,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>gad4</t>
+          <t>gad3</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Trouble relaxing</t>
+          <t>Worrying too much about different things</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -665,12 +657,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>gad5</t>
+          <t>gad4</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Being so restless that it is hard to sit still</t>
+          <t>Trouble relaxing</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -699,12 +691,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>gad6</t>
+          <t>gad5</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Becoming easily annoyed or irritable</t>
+          <t>Being so restless that it is hard to sit still</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -733,12 +725,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>gad7</t>
+          <t>gad6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Feeling afraid as if something awful might happen</t>
+          <t>Becoming easily annoyed or irritable</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -762,32 +754,66 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>calculate</t>
+          <t>select_one likert_main</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>GAD7_anxiety</t>
+          <t>gad7</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>anxiety (sum_coded) - Sum of all items (0-21). Severity: 0-4 minimal, 5-9 mild, 10-14 moderate, 15-21 severe.</t>
+          <t>Feeling afraid as if something awful might happen</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>${gad1} + ${gad2} + ${gad3} + ${gad4} + ${gad5} + ${gad6} + ${gad7}</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>likert</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>calculate</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>GAD7_anxiety</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>anxiety (sum_coded) - Sum of all items (0-21). Severity: 0-4 minimal, 5-9 mild, 10-14 moderate, 15-21 severe.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>${gad1} + ${gad2} + ${gad3} + ${gad4} + ${gad5} + ${gad6} + ${gad7}</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>